<commit_message>
Add Northbridge PDF exports, standardize artifact structure, remove prep guides from public repo
</commit_message>
<xml_diff>
--- a/05-halcyon-ai-governance/artifacts/ai_control_crosswalk.xlsx
+++ b/05-halcyon-ai-governance/artifacts/ai_control_crosswalk.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'AI Control Crosswalk'!$A$1:$J$19</definedName>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Legend!$A$1:$B$7</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Legend!$A$1:$B$9</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Summary!$A$1:$C$9</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -27,12 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="154">
   <si>
     <t xml:space="preserve">HALCYON BENEFITS GROUP — AI GOVERNANCE CONTROL CROSSWALK</t>
   </si>
   <si>
-    <t xml:space="preserve">Sample GRC portfolio artifact | Maps each control objective across NIST AI RMF, ISO/IEC 42001 Annex A, EU AI Act (high-risk obligations), and the existing NIST CSF 2.0 security program | Verify citations against current published texts</t>
+    <t xml:space="preserve">Sample GRC portfolio artifact | Maps each control objective across NIST AI RMF, ISO/IEC 42001 Annex A, EU AI Act as amended by Reg. (EU) 2026/1744, and the existing NIST CSF 2.0 program | Verify citations against current published texts</t>
   </si>
   <si>
     <t xml:space="preserve">Control Domain</t>
@@ -464,7 +464,19 @@
     <t xml:space="preserve">EU AI Act column</t>
   </si>
   <si>
-    <t xml:space="preserve">Cites high-risk obligations (Arts. 9-15) and cross-cutting articles (4, 25, 26, 27, 49, 50, 72, 73, 86). Applicability depends on the system's tier per the inventory. Article numbers reflect the adopted regulation; the May 2026 Digital Omnibus proposal affects timelines, not article structure, but verify before citing.</t>
+    <t xml:space="preserve">Cites high-risk obligations (Arts. 9-15) and cross-cutting articles (4, 25, 26, 27, 49, 50, 72, 73, 86). Applicability depends on the system's tier per the inventory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deadlines, as amended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regulation (EU) 2026/1744 (Digital Omnibus on AI, in force 27 July 2026) moved Annex III standalone high-risk obligations to 2 December 2027 and Annex I embedded systems to 2 August 2028. Article 50 transparency duties were NOT deferred and applied from 2 August 2026. Article 5 prohibitions and GPAI obligations were already in force. The Omnibus changed the article structure only marginally; it changed the calendar substantially.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the deferral means for this crosswalk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sixteen additional months on the high-risk controls. It does not change which controls are needed, and it does not touch the transparency control (row 9), which is already past deadline. Planning that treats the deferral as relief rather than runway will arrive at December 2027 in the same position.</t>
   </si>
   <si>
     <t xml:space="preserve">Implementation status</t>
@@ -1645,7 +1657,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1673,7 +1685,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>144</v>
       </c>
@@ -1681,7 +1693,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
         <v>146</v>
       </c>
@@ -1689,12 +1701,28 @@
         <v>147</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>148</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>149</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>